<commit_message>
Add colour-coded July/August Job Change Alerts workbook; generalise build script
Name-only matches are now accepted only against the import's missing-email
placeholder records; other name hits are listed as possible matches.
Cross-tab duplicates are detected via LinkedIn URL, email, phone+first name
or shared HubSpot record.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -824,7 +824,7 @@
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>SOI email ronen@callblitz.com not in HubSpot; matched by phone; Duplicate: same contact also appears in the July tab</t>
+          <t>Source email ronen@callblitz.com not in HubSpot; matched by phone; Duplicate: same contact also appears in the July tab</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="AA17" s="2" t="inlineStr">
         <is>
-          <t>SOI email dustin@curiocity.media not in HubSpot; matched by phone; Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
+          <t>Source email dustin@curiocity.media not in HubSpot; matched by phone; Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="AA40" s="3" t="inlineStr">
         <is>
-          <t>SOI email russa@createroom.com not in HubSpot; matched by phone</t>
+          <t>Source email russa@createroom.com not in HubSpot; matched by phone</t>
         </is>
       </c>
     </row>
@@ -13096,7 +13096,7 @@
       </c>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>Matched on name only (no email/phone in SOI sheet) - please verify</t>
+          <t>Matched on name only (email/phone not in HubSpot; HubSpot record is the import placeholder) - please verify</t>
         </is>
       </c>
     </row>
@@ -20176,7 +20176,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SOI Work Email vs HubSpot Email + Additional email addresses; then Mobile Phone (last 10 digits); then exact first+last name (only when unique)</t>
+          <t>Source Work Email vs HubSpot Email + Additional email addresses; then Mobile Phone (last 10 digits); then exact first+last name (only when unique AND the HubSpot record is the missing-email import placeholder; other name hits are listed as possible matches, uncoloured)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add colour-coded July/August Speed Dating workbook; extend matching
- Column aliases and explicit source tab names so any import list works
- Name-only matches verified by import placeholder, the list's campaign
  utm_campaign, or email domain vs company; unverified hits listed as
  possible matches
- Rows without email/phone borrow the HubSpot match of another row with
  the same LinkedIn URL/email

SOI and JCA workbooks rebuilt; their results are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -13096,7 +13096,7 @@
       </c>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>Matched on name only (email/phone not in HubSpot; HubSpot record is the import placeholder) - please verify</t>
+          <t>Matched on name only, verified by import placeholder / campaign utm / email domain vs company - please verify</t>
         </is>
       </c>
     </row>
@@ -20176,7 +20176,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Source Work Email vs HubSpot Email + Additional email addresses; then Mobile Phone (last 10 digits); then exact first+last name (only when unique AND the HubSpot record is the missing-email import placeholder; other name hits are listed as possible matches, uncoloured)</t>
+          <t>Source Work Email vs HubSpot Email + Additional email addresses; then Mobile Phone (last 10 digits); then the match of another row in the workbook with the same LinkedIn URL/email; then exact first+last name, accepted only when verified (HubSpot record is the missing-email import placeholder, carries this list's campaign utm_campaign, or its email domain matches the contact's company/domain); unverified name hits are listed as possible matches, uncoloured</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Widen Brown rule: any non-blank utm, blank deal stage, expanded lead statuses
Brown now covers Not a Fit, Cancelled, Unqualified, Attempted to Contact,
Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture and Invalid
Contact Info, with no task requirement. All three workbooks rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +86,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7032,57 +7035,57 @@
       <c r="Y4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Joy</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Stark-Smith</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Vice President Marketing</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>joy.stark-smith@agilityrobotics.com</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>16173083306</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/ACoAAACNGkABT-A8VGo1HrR9lV29bOnwY7q-Pag</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Agility Robotics</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>agilityrobotics.com</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Boston, Massachusetts, United States</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Cengage Learning</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>AI Research SOI Campaign for Joy Stark-Smith
 Lead: Joy Stark-Smith
@@ -7228,56 +7231,56 @@
 Thanks, Joy.”</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>223240411011</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Joy Stark-Smith</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>joy.stark-smith@agilityrobotics.com</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>No Response</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>sphere_of_influence</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="n">
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="n">
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr"/>
+      <c r="W5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -15671,7 +15674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q71"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15842,77 +15845,77 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Ronen R.</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Pessar</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Co-Founder</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>ronen@callblitz.com</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>+12162257700</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/ACoAAAwcjW4BvCJUAK0fWiSBca-E80oRWsQF_oI</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Outbound Operators</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>248860170873</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>sphere_of_influence</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr"/>
-      <c r="N3" s="5" t="n">
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="5" t="n">
+      <c r="O3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>Duplicate: same contact also appears in the July tab</t>
         </is>
@@ -16220,77 +16223,77 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Shana</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Glenzer</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>VP Marketing</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>shana.glenzer@haast.io</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>+12024132352</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/ACoAAADeiokBDRlqEsrdFaX2dPXUldZtWSU9VXQ</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Haast</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>247450948513</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Open Deal</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>SAL - Sales Accepted Lead</t>
         </is>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="N9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="6" t="n">
+      <c r="O9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="P9" s="6" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
+      <c r="Q9" s="7" t="inlineStr">
         <is>
           <t>Duplicate in HubSpot: also matches 136183611921 (Shana Glenzer Glenzer, shana@oleria.com, Converted, CSP - Past Customer)</t>
         </is>
@@ -16537,77 +16540,77 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Hannah</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Swanson</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Vice President Marketing</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>hannah.swanson@rsvpify.com</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>+14012413051</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/hannahswanson</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>RSVPify</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>248860180582</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>sphere_of_influence</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="n">
+      <c r="M14" s="6" t="inlineStr"/>
+      <c r="N14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O14" s="5" t="n">
+      <c r="O14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P14" s="6" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="Q14" s="5" t="inlineStr">
+      <c r="Q14" s="6" t="inlineStr">
         <is>
           <t>Duplicate in HubSpot: also matches 170707734845 (Hannah Swanson, hannah.swanson@intentsify.io, Converted)</t>
         </is>
@@ -16804,7 +16807,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>In HubSpot but does not meet colour criteria: utm_campaign is blank; no upcoming or previous tasks; lead status 'Cold Lead' is not in the Blue or Brown lists | Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
+          <t>In HubSpot but does not meet colour criteria: utm_campaign is blank | Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
       </c>
     </row>
@@ -19795,77 +19798,77 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>July</t>
         </is>
       </c>
-      <c r="B68" s="5" t="n">
+      <c r="B68" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>Ronen R.</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Pessar</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>Co-Founder</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>rp@outboundoperators.com</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>12162257700</t>
         </is>
       </c>
-      <c r="H68" s="5" t="inlineStr">
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/rpessar</t>
         </is>
       </c>
-      <c r="I68" s="5" t="inlineStr">
+      <c r="I68" s="6" t="inlineStr">
         <is>
           <t>Outbound Operators</t>
         </is>
       </c>
-      <c r="J68" s="5" t="inlineStr">
+      <c r="J68" s="6" t="inlineStr">
         <is>
           <t>248860170873</t>
         </is>
       </c>
-      <c r="K68" s="5" t="inlineStr">
+      <c r="K68" s="6" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="L68" s="5" t="inlineStr">
+      <c r="L68" s="6" t="inlineStr">
         <is>
           <t>sphere_of_influence</t>
         </is>
       </c>
-      <c r="M68" s="5" t="inlineStr"/>
-      <c r="N68" s="5" t="n">
+      <c r="M68" s="6" t="inlineStr"/>
+      <c r="N68" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O68" s="5" t="n">
+      <c r="O68" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P68" s="5" t="inlineStr">
+      <c r="P68" s="6" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="Q68" s="5" t="inlineStr">
+      <c r="Q68" s="6" t="inlineStr">
         <is>
           <t>Duplicate: same contact also appears in the August tab</t>
         </is>
@@ -19878,51 +19881,47 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Yannick</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Stark-Smith</t>
+          <t>Selg</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Vice President Marketing</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>joy.stark-smith@agilityrobotics.com</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>16173083306</t>
-        </is>
-      </c>
+          <t>y.selg@autonomyware.ai</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ACoAAACNGkABT-A8VGo1HrR9lV29bOnwY7q-Pag</t>
+          <t>https://www.linkedin.com/in/yannick-selg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Agility Robotics</t>
+          <t>Autonomyware</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>223240411011</t>
+          <t>248860170893</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>No Response</t>
+          <t>New</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -19935,7 +19934,7 @@
         <v>0</v>
       </c>
       <c r="O69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P69" t="inlineStr">
         <is>
@@ -19944,7 +19943,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>In HubSpot but does not meet colour criteria: lead status 'No Response' is not in the Blue or Brown lists</t>
+          <t>In HubSpot but does not meet colour criteria: no upcoming or previous tasks</t>
         </is>
       </c>
     </row>
@@ -19955,42 +19954,38 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Yannick</t>
+          <t>Pramod Abhiram</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Selg</t>
+          <t>Mutyala</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>y.selg@autonomyware.ai</t>
-        </is>
-      </c>
+          <t>Founder &amp; President — Niyantra Robotics Club</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yannick-selg</t>
+          <t>https://www.linkedin.com/in/ACwAAEaXtrUBZKrs5fmJx25O_UY5MSQ1SP8GEQU</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Autonomyware</t>
+          <t>Niyantra Robotics Club DIET</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>248860170893</t>
+          <t>248852134808</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -20016,75 +20011,6 @@
         </is>
       </c>
       <c r="Q70" t="inlineStr">
-        <is>
-          <t>In HubSpot but does not meet colour criteria: no upcoming or previous tasks</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>July</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>28</v>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Pramod Abhiram</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Mutyala</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Founder &amp; President — Niyantra Robotics Club</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ACwAAEaXtrUBZKrs5fmJx25O_UY5MSQ1SP8GEQU</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Niyantra Robotics Club DIET</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>248852134808</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>sphere_of_influence</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="n">
-        <v>0</v>
-      </c>
-      <c r="O71" t="n">
-        <v>0</v>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Q71" t="inlineStr">
         <is>
           <t>In HubSpot but does not meet colour criteria: no upcoming or previous tasks</t>
         </is>
@@ -20109,19 +20035,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Rule applied</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
@@ -20133,19 +20059,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>utm_campaign not blank AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified} AND contact has a previous task</t>
+          <t>utm_campaign not blank (speed_dating or any other value) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info} (no task requirement)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
@@ -20169,7 +20095,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Matching</t>
         </is>
@@ -20205,7 +20131,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
@@ -20260,13 +20186,13 @@
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Brown rule: ignore utm_campaign; rebuild workbooks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -93,8 +93,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1945,109 +1945,109 @@
       <c r="AA16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Dustin is a media executive and strategist working at the intersection of editorial, audience, and revenue, with a focus on building sustainable digital media businesses in an increasingly volatile platform landscape. He specializes in translating complex systems — from content strategy to sales structures and monetization models — into clear, scalable frameworks that align creative ambition with commercial reality. With a background spanning digital publishing, brand partnerships, and organizational design, Dustin is known for his systems thinking, data-informed judgment, and ability to navigate ambiguity while driving growth. He spends most of his time redesigning how modern media actually works — usually one hard conversation and one spreadsheet at a time.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>zdn.ca</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>Toronto, Ontario, Canada</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr"/>
+      <c r="M17" s="5" t="inlineStr"/>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="P17" s="5" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>Dustin Titus</t>
         </is>
       </c>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr">
         <is>
           <t>dustin.titus@gmail.com</t>
         </is>
       </c>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="S17" s="5" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr"/>
-      <c r="U17" s="2" t="inlineStr"/>
-      <c r="V17" s="2" t="n">
+      <c r="T17" s="5" t="inlineStr"/>
+      <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W17" s="2" t="inlineStr"/>
-      <c r="X17" s="2" t="inlineStr"/>
-      <c r="Y17" s="2" t="n">
+      <c r="W17" s="5" t="inlineStr"/>
+      <c r="X17" s="5" t="inlineStr"/>
+      <c r="Y17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AA17" s="2" t="inlineStr">
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="AA17" s="5" t="inlineStr">
         <is>
           <t>Source email dustin@curiocity.media not in HubSpot; matched by phone; Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
@@ -16739,75 +16739,75 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
+      <c r="L17" s="8" t="inlineStr"/>
+      <c r="M17" s="8" t="inlineStr"/>
+      <c r="N17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>In HubSpot but does not meet colour criteria: utm_campaign is blank | Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
       </c>
     </row>
@@ -20035,12 +20035,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Rule applied</t>
         </is>
@@ -20059,14 +20059,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>utm_campaign not blank (speed_dating or any other value) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info} (no task requirement)</t>
+          <t>utm_campaign ignored (any value, including blank) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info} (no task requirement)</t>
         </is>
       </c>
     </row>
@@ -20095,7 +20095,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Matching</t>
         </is>
@@ -20131,7 +20131,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
@@ -20167,13 +20167,13 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Brown rule: require non-blank utm again, add Do Not Contact, ignore tasks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -93,8 +93,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1945,109 +1945,109 @@
       <c r="AA16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Dustin is a media executive and strategist working at the intersection of editorial, audience, and revenue, with a focus on building sustainable digital media businesses in an increasingly volatile platform landscape. He specializes in translating complex systems — from content strategy to sales structures and monetization models — into clear, scalable frameworks that align creative ambition with commercial reality. With a background spanning digital publishing, brand partnerships, and organizational design, Dustin is known for his systems thinking, data-informed judgment, and ability to navigate ambiguity while driving growth. He spends most of his time redesigning how modern media actually works — usually one hard conversation and one spreadsheet at a time.</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>zdn.ca</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Toronto, Ontario, Canada</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr"/>
-      <c r="M17" s="5" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O17" s="5" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="Q17" s="5" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>Dustin Titus</t>
         </is>
       </c>
-      <c r="R17" s="5" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>dustin.titus@gmail.com</t>
         </is>
       </c>
-      <c r="S17" s="5" t="inlineStr">
+      <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="T17" s="5" t="inlineStr"/>
-      <c r="U17" s="5" t="inlineStr"/>
-      <c r="V17" s="5" t="n">
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="W17" s="5" t="inlineStr"/>
-      <c r="X17" s="5" t="inlineStr"/>
-      <c r="Y17" s="5" t="n">
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr"/>
+      <c r="Y17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="Z17" s="5" t="inlineStr">
-        <is>
-          <t>Brown</t>
-        </is>
-      </c>
-      <c r="AA17" s="5" t="inlineStr">
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
         <is>
           <t>Source email dustin@curiocity.media not in HubSpot; matched by phone; Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
@@ -16739,75 +16739,75 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" t="n">
         <v>17</v>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr"/>
-      <c r="M17" s="8" t="inlineStr"/>
-      <c r="N17" s="8" t="n">
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
         <v>0</v>
       </c>
-      <c r="O17" s="8" t="n">
+      <c r="O17" t="n">
         <v>0</v>
       </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>Brown</t>
-        </is>
-      </c>
-      <c r="Q17" s="8" t="inlineStr">
-        <is>
-          <t>Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>In HubSpot but does not meet colour criteria: utm_campaign is blank | Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
       </c>
     </row>
@@ -20035,12 +20035,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Rule applied</t>
         </is>
@@ -20059,14 +20059,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>utm_campaign ignored (any value, including blank) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info} (no task requirement)</t>
+          <t>utm_campaign not blank (speed_dating or any other value) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info, Do Not Contact} (tasks ignored)</t>
         </is>
       </c>
     </row>
@@ -20095,7 +20095,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Matching</t>
         </is>
@@ -20131,7 +20131,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
@@ -20167,13 +20167,13 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Brown rule: ignore utm_campaign and tasks; keep Do Not Contact
Brown = blank deal stage AND lead status in the Brown list, regardless of
utm_campaign (blank allowed) or upcoming/previous tasks (none allowed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W8rSaNPrkh8JAzauZrvbL4
</commit_message>
<xml_diff>
--- a/SOI_July_August_HubSpot_Colour_Coded.xlsx
+++ b/SOI_July_August_HubSpot_Colour_Coded.xlsx
@@ -93,8 +93,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1945,109 +1945,109 @@
       <c r="AA16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Dustin is a media executive and strategist working at the intersection of editorial, audience, and revenue, with a focus on building sustainable digital media businesses in an increasingly volatile platform landscape. He specializes in translating complex systems — from content strategy to sales structures and monetization models — into clear, scalable frameworks that align creative ambition with commercial reality. With a background spanning digital publishing, brand partnerships, and organizational design, Dustin is known for his systems thinking, data-informed judgment, and ability to navigate ambiguity while driving growth. He spends most of his time redesigning how modern media actually works — usually one hard conversation and one spreadsheet at a time.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>zdn.ca</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>Toronto, Ontario, Canada</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr"/>
+      <c r="M17" s="5" t="inlineStr"/>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="P17" s="5" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>Dustin Titus</t>
         </is>
       </c>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr">
         <is>
           <t>dustin.titus@gmail.com</t>
         </is>
       </c>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="S17" s="5" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr"/>
-      <c r="U17" s="2" t="inlineStr"/>
-      <c r="V17" s="2" t="n">
+      <c r="T17" s="5" t="inlineStr"/>
+      <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W17" s="2" t="inlineStr"/>
-      <c r="X17" s="2" t="inlineStr"/>
-      <c r="Y17" s="2" t="n">
+      <c r="W17" s="5" t="inlineStr"/>
+      <c r="X17" s="5" t="inlineStr"/>
+      <c r="Y17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AA17" s="2" t="inlineStr">
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="AA17" s="5" t="inlineStr">
         <is>
           <t>Source email dustin@curiocity.media not in HubSpot; matched by phone; Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
@@ -16739,75 +16739,75 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Dustin</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Chief Revenue Officer (CRO), Digital</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>dustin@curiocity.media</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>+14166254417</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/dustintitus</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Zoomer Media</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>64474598177</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>Cold Lead</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
+      <c r="L17" s="8" t="inlineStr"/>
+      <c r="M17" s="8" t="inlineStr"/>
+      <c r="N17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>In HubSpot but does not meet colour criteria: utm_campaign is blank | Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Duplicate in HubSpot: also matches 47651 (Dustin Titus, dustin@zoomermedia.ca, Cold Lead)</t>
         </is>
       </c>
     </row>
@@ -20035,12 +20035,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Rule applied</t>
         </is>
@@ -20059,14 +20059,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>utm_campaign not blank (speed_dating or any other value) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info, Do Not Contact} (tasks ignored)</t>
+          <t>utm_campaign ignored (any value, including blank) AND upcoming/previous tasks ignored (may be none) AND deal stage blank AND lead status in {Not a Fit, Cancelled, Unqualified, Attempted to Contact, Bad Timing, No Response, No Show, Cold Lead, Long Term Nurture, Invalid Contact Info, Do Not Contact}</t>
         </is>
       </c>
     </row>
@@ -20095,7 +20095,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Matching</t>
         </is>
@@ -20131,7 +20131,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
@@ -20167,13 +20167,13 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">

</xml_diff>